<commit_message>
Review required for Akshata
</commit_message>
<xml_diff>
--- a/output/Etihad Airways/Maharashtra/Apr 26/IMS_OS_all_R1_CDNR_27AABCE6624L1ZG_03062026.xlsx
+++ b/output/Etihad Airways/Maharashtra/Apr 26/IMS_OS_all_R1_CDNR_27AABCE6624L1ZG_03062026.xlsx
@@ -1,141 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\Code\checking rejected credit note\GST-Rejected-Credit-Note-Downloader\output\Etihad Airways\Maharashtra\Apr 26\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12255E37-9761-4788-8562-B6D7E01082B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="16608" windowHeight="8712" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
   <sheets>
     <sheet name="Table 9B" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Table 9B'!$A$5:$P$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Table 9B'!A5:P10</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
-  <si>
-    <t>Goods and Services Tax  - IMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9B - Credit / Debit Notes (Registered)
-</t>
-  </si>
-  <si>
-    <t>Recipient GSTIN</t>
-  </si>
-  <si>
-    <t>Trade/Legal Name</t>
-  </si>
-  <si>
-    <t>Note Number</t>
-  </si>
-  <si>
-    <t>Note Date</t>
-  </si>
-  <si>
-    <t>Note Type</t>
-  </si>
-  <si>
-    <t>Note Supply Type</t>
-  </si>
-  <si>
-    <t>Note Value (₹)</t>
-  </si>
-  <si>
-    <t>Total Taxable Value (₹)</t>
-  </si>
-  <si>
-    <t>Integrated Tax (₹)</t>
-  </si>
-  <si>
-    <t>Central Tax (₹)</t>
-  </si>
-  <si>
-    <t>State/UT Tax (₹)</t>
-  </si>
-  <si>
-    <t>Cess (₹)</t>
-  </si>
-  <si>
-    <t>Return Period</t>
-  </si>
-  <si>
-    <t>Reported in Form</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Remarks by Recipient</t>
-  </si>
-  <si>
-    <t>24AAQPJ7752G1ZF</t>
-  </si>
-  <si>
-    <t>R.A.Dye Chem</t>
-  </si>
-  <si>
-    <t>CN/MH/APR26/5068</t>
-  </si>
-  <si>
-    <t>Credit</t>
-  </si>
-  <si>
-    <t>Regular</t>
-  </si>
-  <si>
-    <t>GSTR-1/IFF</t>
-  </si>
-  <si>
-    <t>Rejected</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>CN/MH/APR26/5067</t>
-  </si>
-  <si>
-    <t>27AAACB2125N1ZS</t>
-  </si>
-  <si>
-    <t>BEACON INDUSTRIAL ELECTRONICS PVT LTD</t>
-  </si>
-  <si>
-    <t>CN/MH/APR26/2861</t>
-  </si>
-  <si>
-    <t>No remarks available</t>
-  </si>
-  <si>
-    <t>27AAACP2029H1ZO</t>
-  </si>
-  <si>
-    <t>PRISM ENGINEERING PVT LTD</t>
-  </si>
-  <si>
-    <t>CN/MH/APR26/6573</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="2">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="60" formatCode="dd-mm-yyyy"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -165,8 +69,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -174,14 +78,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -506,91 +402,88 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P10"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="4" max="4" width="11.3984375" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Goods and Services Tax  - IMS</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>1</v>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str" xml:space="preserve">
+        <v xml:space="preserve">9B - Credit / Debit Notes (Registered)
+</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" t="s">
-        <v>5</v>
-      </c>
-      <c r="E5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" t="s">
-        <v>8</v>
-      </c>
-      <c r="H5" t="s">
-        <v>9</v>
-      </c>
-      <c r="I5" t="s">
-        <v>10</v>
-      </c>
-      <c r="J5" t="s">
-        <v>11</v>
-      </c>
-      <c r="K5" t="s">
-        <v>12</v>
-      </c>
-      <c r="L5" t="s">
-        <v>13</v>
-      </c>
-      <c r="M5" t="s">
-        <v>14</v>
-      </c>
-      <c r="N5" t="s">
-        <v>15</v>
-      </c>
-      <c r="O5" t="s">
-        <v>16</v>
-      </c>
-      <c r="P5" t="s">
-        <v>17</v>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Recipient GSTIN</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Trade/Legal Name</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Note Number</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Note Date</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Note Type</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Note Supply Type</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Note Value (₹)</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Total Taxable Value (₹)</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Integrated Tax (₹)</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Central Tax (₹)</v>
+      </c>
+      <c r="K5" t="str">
+        <v>State/UT Tax (₹)</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Cess (₹)</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Return Period</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Reported in Form</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Status</v>
+      </c>
+      <c r="P5" t="str">
+        <v>Remarks by Recipient</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="1">
-        <v>46142.229166666664</v>
-      </c>
-      <c r="E7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" t="s">
-        <v>22</v>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>24AAQPJ7752G1ZF</v>
+      </c>
+      <c r="B7" t="str">
+        <v>R.A.Dye Chem</v>
+      </c>
+      <c r="C7" t="str">
+        <v>CN/MH/APR26/5068</v>
+      </c>
+      <c r="D7" s="1" t="d">
+        <v>2026-04-30T05:30:00.000Z</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Credit</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Regular</v>
       </c>
       <c r="G7">
         <v>53305</v>
@@ -610,37 +503,37 @@
       <c r="L7">
         <v>0</v>
       </c>
-      <c r="M7" s="2">
-        <v>46113.229166666664</v>
-      </c>
-      <c r="N7" t="s">
-        <v>23</v>
-      </c>
-      <c r="O7" t="s">
-        <v>24</v>
-      </c>
-      <c r="P7" t="s">
-        <v>25</v>
+      <c r="M7" s="2" t="d">
+        <v>2026-04-01T05:30:00.000Z</v>
+      </c>
+      <c r="N7" t="str">
+        <v>GSTR-1/IFF</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Rejected</v>
+      </c>
+      <c r="P7" t="str">
+        <v>NA</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="1">
-        <v>46142.229166666664</v>
-      </c>
-      <c r="E8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" t="s">
-        <v>22</v>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>24AAQPJ7752G1ZF</v>
+      </c>
+      <c r="B8" t="str">
+        <v>R.A.Dye Chem</v>
+      </c>
+      <c r="C8" t="str">
+        <v>CN/MH/APR26/5067</v>
+      </c>
+      <c r="D8" s="1" t="d">
+        <v>2026-04-30T05:30:00.000Z</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Credit</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Regular</v>
       </c>
       <c r="G8">
         <v>53305</v>
@@ -660,37 +553,37 @@
       <c r="L8">
         <v>0</v>
       </c>
-      <c r="M8" s="2">
-        <v>46113.229166666664</v>
-      </c>
-      <c r="N8" t="s">
-        <v>23</v>
-      </c>
-      <c r="O8" t="s">
-        <v>24</v>
-      </c>
-      <c r="P8" t="s">
-        <v>25</v>
+      <c r="M8" s="2" t="d">
+        <v>2026-04-01T05:30:00.000Z</v>
+      </c>
+      <c r="N8" t="str">
+        <v>GSTR-1/IFF</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Rejected</v>
+      </c>
+      <c r="P8" t="str">
+        <v>NA</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="1">
-        <v>46142.229166666664</v>
-      </c>
-      <c r="E9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" t="s">
-        <v>22</v>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>27AAACB2125N1ZS</v>
+      </c>
+      <c r="B9" t="str">
+        <v>BEACON INDUSTRIAL ELECTRONICS PVT LTD</v>
+      </c>
+      <c r="C9" t="str">
+        <v>CN/MH/APR26/2861</v>
+      </c>
+      <c r="D9" s="1" t="d">
+        <v>2026-04-30T05:30:00.000Z</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Credit</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Regular</v>
       </c>
       <c r="G9">
         <v>74130</v>
@@ -710,37 +603,37 @@
       <c r="L9">
         <v>0</v>
       </c>
-      <c r="M9" s="2">
-        <v>46113.229166666664</v>
-      </c>
-      <c r="N9" t="s">
-        <v>23</v>
-      </c>
-      <c r="O9" t="s">
-        <v>24</v>
-      </c>
-      <c r="P9" t="s">
-        <v>30</v>
+      <c r="M9" s="2" t="d">
+        <v>2026-04-01T05:30:00.000Z</v>
+      </c>
+      <c r="N9" t="str">
+        <v>GSTR-1/IFF</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Rejected</v>
+      </c>
+      <c r="P9" t="str">
+        <v>No remarks available</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" s="1">
-        <v>46142.229166666664</v>
-      </c>
-      <c r="E10" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" t="s">
-        <v>22</v>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>27AAACP2029H1ZO</v>
+      </c>
+      <c r="B10" t="str">
+        <v>PRISM ENGINEERING PVT LTD</v>
+      </c>
+      <c r="C10" t="str">
+        <v>CN/MH/APR26/6573</v>
+      </c>
+      <c r="D10" s="1" t="d">
+        <v>2026-04-30T05:30:00.000Z</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Credit</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Regular</v>
       </c>
       <c r="G10">
         <v>37812</v>
@@ -760,24 +653,23 @@
       <c r="L10">
         <v>0</v>
       </c>
-      <c r="M10" s="2">
-        <v>46113.229166666664</v>
-      </c>
-      <c r="N10" t="s">
-        <v>23</v>
-      </c>
-      <c r="O10" t="s">
-        <v>24</v>
-      </c>
-      <c r="P10" t="s">
-        <v>30</v>
+      <c r="M10" s="2" t="d">
+        <v>2026-04-01T05:30:00.000Z</v>
+      </c>
+      <c r="N10" t="str">
+        <v>GSTR-1/IFF</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Rejected</v>
+      </c>
+      <c r="P10" t="str">
+        <v>No remarks available</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:P10" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A5:P10"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:P10" numberStoredAsText="1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>